<commit_message>
Update app, models and README
</commit_message>
<xml_diff>
--- a/cluster_analysis.xlsx
+++ b/cluster_analysis.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,122 +466,142 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Heart Disease Stage</t>
+          <t>sex_Female</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>sex_Female</t>
+          <t>sex_Male</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>sex_Male</t>
+          <t>dataset_Cleveland</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>dataset_Cleveland</t>
+          <t>dataset_Hungary</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>dataset_Hungary</t>
+          <t>dataset_Switzerland</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>dataset_Switzerland</t>
+          <t>dataset_VA Long Beach</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>dataset_VA Long Beach</t>
+          <t>cp_asymptomatic</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>cp_asymptomatic</t>
+          <t>cp_atypical angina</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>cp_atypical angina</t>
+          <t>cp_non-anginal</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>cp_non-anginal</t>
+          <t>cp_typical angina</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>cp_typical angina</t>
+          <t>fbs_False</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>fbs_False</t>
+          <t>fbs_True</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>fbs_True</t>
+          <t>restecg_lv hypertrophy</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>restecg_lv hypertrophy</t>
+          <t>restecg_normal</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>restecg_normal</t>
+          <t>restecg_st-t abnormality</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>restecg_st-t abnormality</t>
+          <t>exang_False</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>exang_False</t>
+          <t>exang_True</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>exang_True</t>
+          <t>slope_downsloping</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>slope_downsloping</t>
+          <t>slope_flat</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>slope_flat</t>
+          <t>slope_upsloping</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>slope_upsloping</t>
+          <t>thal_fixed defect</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>thal_fixed defect</t>
+          <t>thal_normal</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>thal_normal</t>
+          <t>thal_reversable defect</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>thal_reversable defect</t>
+          <t>Heart Disease Stage_0</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Heart Disease Stage_1</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Heart Disease Stage_2</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Heart Disease Stage_3</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Heart Disease Stage_4</t>
         </is>
       </c>
     </row>
@@ -590,94 +610,106 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>48.928125</v>
+        <v>52.392</v>
       </c>
       <c r="C2" t="n">
-        <v>129.059375</v>
+        <v>129.608</v>
       </c>
       <c r="D2" t="n">
-        <v>237.515625</v>
+        <v>241.674</v>
       </c>
       <c r="E2" t="n">
-        <v>151.784375</v>
+        <v>159.204</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2934375</v>
+        <v>0.578</v>
       </c>
       <c r="G2" t="n">
-        <v>0.090625</v>
+        <v>0.282</v>
       </c>
       <c r="H2" t="n">
-        <v>0.03125</v>
+        <v>0.431</v>
       </c>
       <c r="I2" t="n">
-        <v>140</v>
+        <v>0.569</v>
       </c>
       <c r="J2" t="n">
-        <v>180</v>
+        <v>0.956</v>
       </c>
       <c r="K2" t="n">
-        <v>131</v>
+        <v>0.028</v>
       </c>
       <c r="L2" t="n">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>0.017</v>
       </c>
       <c r="N2" t="n">
-        <v>15</v>
+        <v>0.232</v>
       </c>
       <c r="O2" t="n">
-        <v>59</v>
+        <v>0.249</v>
       </c>
       <c r="P2" t="n">
-        <v>144</v>
+        <v>0.414</v>
       </c>
       <c r="Q2" t="n">
-        <v>105</v>
+        <v>0.105</v>
       </c>
       <c r="R2" t="n">
-        <v>12</v>
+        <v>0.867</v>
       </c>
       <c r="S2" t="n">
-        <v>310</v>
+        <v>0.133</v>
       </c>
       <c r="T2" t="n">
-        <v>10</v>
+        <v>0.448</v>
       </c>
       <c r="U2" t="n">
-        <v>56</v>
+        <v>0.541</v>
       </c>
       <c r="V2" t="n">
-        <v>229</v>
+        <v>0.011</v>
       </c>
       <c r="W2" t="n">
-        <v>35</v>
+        <v>0.895</v>
       </c>
       <c r="X2" t="n">
-        <v>303</v>
+        <v>0.105</v>
       </c>
       <c r="Y2" t="n">
-        <v>17</v>
+        <v>0.05</v>
       </c>
       <c r="Z2" t="n">
-        <v>5</v>
+        <v>0.249</v>
       </c>
       <c r="AA2" t="n">
-        <v>211</v>
+        <v>0.702</v>
       </c>
       <c r="AB2" t="n">
-        <v>104</v>
+        <v>0.028</v>
       </c>
       <c r="AC2" t="n">
-        <v>5</v>
+        <v>0.834</v>
       </c>
       <c r="AD2" t="n">
-        <v>308</v>
+        <v>0.138</v>
       </c>
       <c r="AE2" t="n">
-        <v>7</v>
+        <v>0.878</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -685,94 +717,106 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>59.03</v>
+        <v>56.943</v>
       </c>
       <c r="C3" t="n">
-        <v>137.97</v>
+        <v>133.566</v>
       </c>
       <c r="D3" t="n">
-        <v>209.13</v>
+        <v>251.516</v>
       </c>
       <c r="E3" t="n">
-        <v>134.39</v>
+        <v>135.721</v>
       </c>
       <c r="F3" t="n">
-        <v>0.885</v>
+        <v>1.753</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04</v>
+        <v>1.23</v>
       </c>
       <c r="H3" t="n">
-        <v>1.33</v>
+        <v>0.139</v>
       </c>
       <c r="I3" t="n">
-        <v>6</v>
+        <v>0.861</v>
       </c>
       <c r="J3" t="n">
-        <v>94</v>
+        <v>0.984</v>
       </c>
       <c r="K3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>4</v>
+        <v>0.016</v>
       </c>
       <c r="N3" t="n">
-        <v>68</v>
+        <v>0.82</v>
       </c>
       <c r="O3" t="n">
-        <v>57</v>
+        <v>0.016</v>
       </c>
       <c r="P3" t="n">
-        <v>11</v>
+        <v>0.123</v>
       </c>
       <c r="Q3" t="n">
-        <v>22</v>
+        <v>0.041</v>
       </c>
       <c r="R3" t="n">
-        <v>10</v>
+        <v>0.836</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>0.164</v>
       </c>
       <c r="T3" t="n">
-        <v>100</v>
+        <v>0.59</v>
       </c>
       <c r="U3" t="n">
-        <v>22</v>
+        <v>0.393</v>
       </c>
       <c r="V3" t="n">
-        <v>36</v>
+        <v>0.016</v>
       </c>
       <c r="W3" t="n">
-        <v>42</v>
+        <v>0.361</v>
       </c>
       <c r="X3" t="n">
-        <v>70</v>
+        <v>0.639</v>
       </c>
       <c r="Y3" t="n">
-        <v>30</v>
+        <v>0.107</v>
       </c>
       <c r="Z3" t="n">
-        <v>11</v>
+        <v>0.705</v>
       </c>
       <c r="AA3" t="n">
-        <v>81</v>
+        <v>0.189</v>
       </c>
       <c r="AB3" t="n">
-        <v>8</v>
+        <v>0.107</v>
       </c>
       <c r="AC3" t="n">
-        <v>9</v>
+        <v>0.131</v>
       </c>
       <c r="AD3" t="n">
-        <v>75</v>
+        <v>0.762</v>
       </c>
       <c r="AE3" t="n">
-        <v>16</v>
+        <v>0.074</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0.107</v>
       </c>
     </row>
     <row r="4">
@@ -780,94 +824,106 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>56.43421052631579</v>
+        <v>57.237</v>
       </c>
       <c r="C4" t="n">
-        <v>133.3947368421053</v>
+        <v>134.836</v>
       </c>
       <c r="D4" t="n">
-        <v>248.3223684210526</v>
+        <v>205.047</v>
       </c>
       <c r="E4" t="n">
-        <v>140.9078947368421</v>
+        <v>125.314</v>
       </c>
       <c r="F4" t="n">
-        <v>1.514473684210526</v>
+        <v>1.223</v>
       </c>
       <c r="G4" t="n">
-        <v>1.105263157894737</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1.736842105263158</v>
+        <v>0.051</v>
       </c>
       <c r="I4" t="n">
-        <v>19</v>
+        <v>0.949</v>
       </c>
       <c r="J4" t="n">
-        <v>133</v>
+        <v>0.026</v>
       </c>
       <c r="K4" t="n">
-        <v>150</v>
+        <v>0.277</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>0.697</v>
       </c>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>0.741</v>
       </c>
       <c r="O4" t="n">
-        <v>107</v>
+        <v>0.051</v>
       </c>
       <c r="P4" t="n">
-        <v>8</v>
+        <v>0.179</v>
       </c>
       <c r="Q4" t="n">
-        <v>23</v>
+        <v>0.029</v>
       </c>
       <c r="R4" t="n">
-        <v>14</v>
+        <v>0.675</v>
       </c>
       <c r="S4" t="n">
-        <v>131</v>
+        <v>0.296</v>
       </c>
       <c r="T4" t="n">
-        <v>21</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="U4" t="n">
-        <v>93</v>
+        <v>0.496</v>
       </c>
       <c r="V4" t="n">
-        <v>57</v>
+        <v>0.416</v>
       </c>
       <c r="W4" t="n">
-        <v>2</v>
+        <v>0.19</v>
       </c>
       <c r="X4" t="n">
-        <v>70</v>
+        <v>0.624</v>
       </c>
       <c r="Y4" t="n">
-        <v>82</v>
+        <v>0.106</v>
       </c>
       <c r="Z4" t="n">
-        <v>14</v>
+        <v>0.847</v>
       </c>
       <c r="AA4" t="n">
-        <v>90</v>
+        <v>0.047</v>
       </c>
       <c r="AB4" t="n">
-        <v>48</v>
+        <v>0.036</v>
       </c>
       <c r="AC4" t="n">
-        <v>14</v>
+        <v>0.876</v>
       </c>
       <c r="AD4" t="n">
-        <v>28</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AE4" t="n">
-        <v>110</v>
+        <v>0.19</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0.036</v>
       </c>
     </row>
     <row r="5">
@@ -875,94 +931,106 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>57.47031963470319</v>
+        <v>46.877</v>
       </c>
       <c r="C5" t="n">
-        <v>130.2831050228311</v>
+        <v>130.555</v>
       </c>
       <c r="D5" t="n">
-        <v>69.53424657534246</v>
+        <v>242.295</v>
       </c>
       <c r="E5" t="n">
-        <v>122.2511415525114</v>
+        <v>145.441</v>
       </c>
       <c r="F5" t="n">
-        <v>0.945662100456621</v>
+        <v>0.236</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0365296803652968</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>1.799086757990868</v>
+        <v>0.341</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>0.659</v>
       </c>
       <c r="J5" t="n">
-        <v>209</v>
+        <v>0.018</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0.964</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>117</v>
+        <v>0.018</v>
       </c>
       <c r="N5" t="n">
-        <v>101</v>
+        <v>0.241</v>
       </c>
       <c r="O5" t="n">
-        <v>167</v>
+        <v>0.495</v>
       </c>
       <c r="P5" t="n">
-        <v>4</v>
+        <v>0.218</v>
       </c>
       <c r="Q5" t="n">
-        <v>42</v>
+        <v>0.045</v>
       </c>
       <c r="R5" t="n">
-        <v>6</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="S5" t="n">
-        <v>218</v>
+        <v>0.036</v>
       </c>
       <c r="T5" t="n">
-        <v>1</v>
+        <v>0.018</v>
       </c>
       <c r="U5" t="n">
-        <v>16</v>
+        <v>0.841</v>
       </c>
       <c r="V5" t="n">
-        <v>127</v>
+        <v>0.141</v>
       </c>
       <c r="W5" t="n">
-        <v>76</v>
+        <v>0.918</v>
       </c>
       <c r="X5" t="n">
-        <v>107</v>
+        <v>0.068</v>
       </c>
       <c r="Y5" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>32</v>
+        <v>0.968</v>
       </c>
       <c r="AA5" t="n">
-        <v>144</v>
+        <v>0.032</v>
       </c>
       <c r="AB5" t="n">
-        <v>43</v>
+        <v>0.036</v>
       </c>
       <c r="AC5" t="n">
-        <v>12</v>
+        <v>0.927</v>
       </c>
       <c r="AD5" t="n">
-        <v>159</v>
+        <v>0.036</v>
       </c>
       <c r="AE5" t="n">
-        <v>48</v>
+        <v>0.832</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -970,94 +1038,106 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>50.43410852713178</v>
+        <v>55.317</v>
       </c>
       <c r="C6" t="n">
-        <v>135.906976744186</v>
+        <v>130.203</v>
       </c>
       <c r="D6" t="n">
-        <v>263.7596899224806</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>127.7209302325581</v>
+        <v>121.707</v>
       </c>
       <c r="F6" t="n">
-        <v>1.281395348837209</v>
+        <v>0.646</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>0.065</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8914728682170543</v>
+        <v>0.081</v>
       </c>
       <c r="I6" t="n">
-        <v>19</v>
+        <v>0.919</v>
       </c>
       <c r="J6" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>109</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>14</v>
+        <v>0.797</v>
       </c>
       <c r="O6" t="n">
-        <v>106</v>
+        <v>0.033</v>
       </c>
       <c r="P6" t="n">
-        <v>7</v>
+        <v>0.138</v>
       </c>
       <c r="Q6" t="n">
-        <v>12</v>
+        <v>0.033</v>
       </c>
       <c r="R6" t="n">
-        <v>4</v>
+        <v>0.35</v>
       </c>
       <c r="S6" t="n">
-        <v>123</v>
+        <v>0.041</v>
       </c>
       <c r="T6" t="n">
-        <v>6</v>
+        <v>0.057</v>
       </c>
       <c r="U6" t="n">
-        <v>1</v>
+        <v>0.699</v>
       </c>
       <c r="V6" t="n">
-        <v>104</v>
+        <v>0.244</v>
       </c>
       <c r="W6" t="n">
-        <v>24</v>
+        <v>0.553</v>
       </c>
       <c r="X6" t="n">
-        <v>33</v>
+        <v>0.439</v>
       </c>
       <c r="Y6" t="n">
-        <v>96</v>
+        <v>0.098</v>
       </c>
       <c r="Z6" t="n">
-        <v>1</v>
+        <v>0.634</v>
       </c>
       <c r="AA6" t="n">
-        <v>128</v>
+        <v>0.268</v>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>0.081</v>
       </c>
       <c r="AC6" t="n">
-        <v>6</v>
+        <v>0.577</v>
       </c>
       <c r="AD6" t="n">
-        <v>112</v>
+        <v>0.341</v>
       </c>
       <c r="AE6" t="n">
-        <v>11</v>
+        <v>0.065</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0.244</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0.041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>